<commit_message>
Polish CapitalOps evidence workbook layout
</commit_message>
<xml_diff>
--- a/projects/capitalops/downloads/CapitalOps_Source_Evidence_Pack.xlsx
+++ b/projects/capitalops/downloads/CapitalOps_Source_Evidence_Pack.xlsx
@@ -2,20 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="START HERE" sheetId="1" r:id="Rf778100f1da542c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INVESTIGATION LOG" sheetId="2" r:id="R30168501845643b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TRIAL BALANCE" sheetId="3" r:id="Rfd570f5891604239"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BANK STATEMENT" sheetId="4" r:id="Rdac8a1a48f204555"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASH GL" sheetId="5" r:id="Rc5ff2ca46c754f35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BANK SUPPORT" sheetId="6" r:id="R31bc5cccee0840a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP GL" sheetId="7" r:id="Rbda5f32ae8cf4f68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP SUBLEDGER" sheetId="8" r:id="R72a40330ee6b408a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EXPENSE DETAIL" sheetId="9" r:id="Rbb0076039f98446d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FA REGISTER" sheetId="10" r:id="Rc9a010de7d0b4b1f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DISPOSAL LOG" sheetId="11" r:id="Ra867b3d2821243bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DEPRECIATION RUN" sheetId="12" r:id="R6ea057118ed44b06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PREPAIDS &amp; ACCRUALS" sheetId="13" r:id="Ra4d67db5601e426e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="POLICY &amp; SOURCE MAP" sheetId="14" r:id="R30ec1cc2c90b4420"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="START HERE" sheetId="1" r:id="R5bb4e104d6604735"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INVESTIGATION LOG" sheetId="2" r:id="R3a89cd7e675349ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TRIAL BALANCE" sheetId="3" r:id="R77847113f7464dc7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BANK STATEMENT" sheetId="4" r:id="R9c9bce7adf044a72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CASH GL" sheetId="5" r:id="R98040ebad9144400"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BANK SUPPORT" sheetId="6" r:id="R5d78d4e1524d42e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP GL" sheetId="7" r:id="R929e2b34d5f9408d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AP SUBLEDGER" sheetId="8" r:id="Ra071505dc0c64592"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EXPENSE DETAIL" sheetId="9" r:id="Rfbacd359a15141fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FA REGISTER" sheetId="10" r:id="Ra840bf3f13644680"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DISPOSAL LOG" sheetId="11" r:id="R4ac3bf549bb641f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DEPRECIATION RUN" sheetId="12" r:id="R40e204f12ebd415a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PREPAIDS &amp; ACCRUALS" sheetId="13" r:id="R576fe676d7cd424c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="POLICY &amp; SOURCE MAP" sheetId="14" r:id="Rd5e3765e224b4ae5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -147,7 +147,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="49">
+  <x:cellXfs count="54">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -255,6 +255,21 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1194,12 +1209,12 @@
         <x:f>E5-F5</x:f>
         <x:v>2000000</x:v>
       </x:c>
-      <x:c r="H5" s="28" t="str">
+      <x:c r="H5" s="49" t="str">
         <x:v>Active</x:v>
       </x:c>
-      <x:c r="I5" s="28"/>
-      <x:c r="J5" s="28"/>
-      <x:c r="K5" s="28" t="n">
+      <x:c r="I5" s="49"/>
+      <x:c r="J5" s="49"/>
+      <x:c r="K5" s="49" t="n">
         <x:f>COUNTIF('DISPOSAL LOG'!$A$5:$A$12,A5)</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -1231,16 +1246,16 @@
         <x:f>E6-F6</x:f>
         <x:v>5000000</x:v>
       </x:c>
-      <x:c r="H6" s="28" t="str">
+      <x:c r="H6" s="49" t="str">
         <x:v>Active</x:v>
       </x:c>
-      <x:c r="I6" s="28" t="n">
+      <x:c r="I6" s="49" t="n">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="J6" s="28" t="n">
+      <x:c r="J6" s="49" t="n">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="K6" s="28" t="n">
+      <x:c r="K6" s="49" t="n">
         <x:f>COUNTIF('DISPOSAL LOG'!$A$5:$A$12,A6)</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -1272,16 +1287,16 @@
         <x:f>E7-F7</x:f>
         <x:v>1300000</x:v>
       </x:c>
-      <x:c r="H7" s="28" t="str">
+      <x:c r="H7" s="49" t="str">
         <x:v>Active</x:v>
       </x:c>
-      <x:c r="I7" s="28" t="n">
+      <x:c r="I7" s="49" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="J7" s="28" t="n">
+      <x:c r="J7" s="49" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="K7" s="28" t="n">
+      <x:c r="K7" s="49" t="n">
         <x:f>COUNTIF('DISPOSAL LOG'!$A$5:$A$12,A7)</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -1313,16 +1328,16 @@
         <x:f>E8-F8</x:f>
         <x:v>114510</x:v>
       </x:c>
-      <x:c r="H8" s="28" t="str">
+      <x:c r="H8" s="49" t="str">
         <x:v>Active</x:v>
       </x:c>
-      <x:c r="I8" s="28" t="n">
+      <x:c r="I8" s="49" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="J8" s="28" t="n">
+      <x:c r="J8" s="49" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="K8" s="28" t="n">
+      <x:c r="K8" s="49" t="n">
         <x:f>COUNTIF('DISPOSAL LOG'!$A$5:$A$12,A8)</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -1354,16 +1369,16 @@
         <x:f>E9-F9</x:f>
         <x:v>18600</x:v>
       </x:c>
-      <x:c r="H9" s="28" t="str">
+      <x:c r="H9" s="49" t="str">
         <x:v>Active</x:v>
       </x:c>
-      <x:c r="I9" s="28" t="n">
+      <x:c r="I9" s="49" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="J9" s="28" t="n">
+      <x:c r="J9" s="49" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="K9" s="28" t="n">
+      <x:c r="K9" s="49" t="n">
         <x:f>COUNTIF('DISPOSAL LOG'!$A$5:$A$12,A9)</x:f>
         <x:v>1</x:v>
       </x:c>
@@ -1395,16 +1410,16 @@
         <x:f>E10-F10</x:f>
         <x:v>112300</x:v>
       </x:c>
-      <x:c r="H10" s="28" t="str">
+      <x:c r="H10" s="49" t="str">
         <x:v>Active</x:v>
       </x:c>
-      <x:c r="I10" s="28" t="n">
+      <x:c r="I10" s="49" t="n">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="J10" s="28" t="n">
+      <x:c r="J10" s="49" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="K10" s="28" t="n">
+      <x:c r="K10" s="49" t="n">
         <x:f>COUNTIF('DISPOSAL LOG'!$A$5:$A$12,A10)</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -1436,16 +1451,16 @@
         <x:f>E11-F11</x:f>
         <x:v>1278000</x:v>
       </x:c>
-      <x:c r="H11" s="17" t="str">
+      <x:c r="H11" s="50" t="str">
         <x:v>Active</x:v>
       </x:c>
-      <x:c r="I11" s="17" t="n">
+      <x:c r="I11" s="50" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="J11" s="17" t="n">
+      <x:c r="J11" s="50" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="K11" s="17" t="n">
+      <x:c r="K11" s="50" t="n">
         <x:f>COUNTIF('DISPOSAL LOG'!$A$5:$A$12,A11)</x:f>
         <x:v>0</x:v>
       </x:c>
@@ -1630,16 +1645,16 @@
       <x:c r="E5" s="44" t="n">
         <x:v>51400</x:v>
       </x:c>
-      <x:c r="F5" s="44" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G5" s="17" t="str">
+      <x:c r="F5" s="51" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G5" s="50" t="str">
         <x:v>Approved</x:v>
       </x:c>
-      <x:c r="H5" s="17" t="str">
+      <x:c r="H5" s="50" t="str">
         <x:v>Released to recycler</x:v>
       </x:c>
-      <x:c r="I5" s="17" t="str">
+      <x:c r="I5" s="50" t="str">
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="J5" s="17" t="str">
@@ -1795,13 +1810,13 @@
       <x:c r="D5" s="43" t="n">
         <x:v>1278000</x:v>
       </x:c>
-      <x:c r="E5" s="28" t="n">
+      <x:c r="E5" s="49" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="F5" s="28" t="n">
+      <x:c r="F5" s="49" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G5" s="28" t="str">
+      <x:c r="G5" s="49" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="H5" s="43" t="n">
@@ -1815,7 +1830,7 @@
         <x:f>I5-H5</x:f>
         <x:v>21300</x:v>
       </x:c>
-      <x:c r="K5" s="28" t="str">
+      <x:c r="K5" s="49" t="str">
         <x:f>IF(AND(C5&lt;=DATE(2026,4,30),G5="No"),"REVIEW","CLEAR")</x:f>
         <x:v>REVIEW</x:v>
       </x:c>
@@ -1837,13 +1852,13 @@
       <x:c r="D6" s="43" t="n">
         <x:v>132300</x:v>
       </x:c>
-      <x:c r="E6" s="28" t="n">
+      <x:c r="E6" s="49" t="n">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="F6" s="28" t="n">
+      <x:c r="F6" s="49" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G6" s="28" t="str">
+      <x:c r="G6" s="49" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="H6" s="43" t="n">
@@ -1857,7 +1872,7 @@
         <x:f>I6-H6</x:f>
         <x:v>1470</x:v>
       </x:c>
-      <x:c r="K6" s="28" t="str">
+      <x:c r="K6" s="49" t="str">
         <x:f>IF(AND(C6&lt;=DATE(2026,4,30),G6="No"),"REVIEW","CLEAR")</x:f>
         <x:v>CLEAR</x:v>
       </x:c>
@@ -1879,13 +1894,13 @@
       <x:c r="D7" s="44" t="n">
         <x:v>319700</x:v>
       </x:c>
-      <x:c r="E7" s="17" t="n">
+      <x:c r="E7" s="50" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="F7" s="17" t="n">
+      <x:c r="F7" s="50" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="G7" s="17" t="str">
+      <x:c r="G7" s="50" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="H7" s="44" t="n">
@@ -1899,7 +1914,7 @@
         <x:f>I7-H7</x:f>
         <x:v>0.33333333333303017</x:v>
       </x:c>
-      <x:c r="K7" s="17" t="str">
+      <x:c r="K7" s="50" t="str">
         <x:f>IF(AND(C7&lt;=DATE(2026,4,30),G7="No"),"REVIEW","CLEAR")</x:f>
         <x:v>CLEAR</x:v>
       </x:c>
@@ -2442,7 +2457,7 @@
       <x:c r="E6" s="28" t="str">
         <x:v>Controller</x:v>
       </x:c>
-      <x:c r="F6" s="46" t="n">
+      <x:c r="F6" s="52" t="n">
         <x:v>46023</x:v>
       </x:c>
       <x:c r="G6" s="28" t="str">
@@ -2468,7 +2483,7 @@
       <x:c r="E7" s="28" t="str">
         <x:v>Controller</x:v>
       </x:c>
-      <x:c r="F7" s="46" t="n">
+      <x:c r="F7" s="52" t="n">
         <x:v>46023</x:v>
       </x:c>
       <x:c r="G7" s="28" t="str">
@@ -2494,7 +2509,7 @@
       <x:c r="E8" s="28" t="str">
         <x:v>Controller</x:v>
       </x:c>
-      <x:c r="F8" s="46" t="n">
+      <x:c r="F8" s="52" t="n">
         <x:v>46023</x:v>
       </x:c>
       <x:c r="G8" s="28" t="str">
@@ -2520,7 +2535,7 @@
       <x:c r="E9" s="28" t="str">
         <x:v>Controller</x:v>
       </x:c>
-      <x:c r="F9" s="46" t="n">
+      <x:c r="F9" s="52" t="n">
         <x:v>46023</x:v>
       </x:c>
       <x:c r="G9" s="28" t="str">
@@ -2546,7 +2561,7 @@
       <x:c r="E10" s="28" t="str">
         <x:v>Controller</x:v>
       </x:c>
-      <x:c r="F10" s="46" t="n">
+      <x:c r="F10" s="52" t="n">
         <x:v>46023</x:v>
       </x:c>
       <x:c r="G10" s="28" t="str">
@@ -2572,7 +2587,7 @@
       <x:c r="E11" s="17" t="str">
         <x:v>CFO</x:v>
       </x:c>
-      <x:c r="F11" s="47" t="n">
+      <x:c r="F11" s="53" t="n">
         <x:v>46023</x:v>
       </x:c>
       <x:c r="G11" s="17" t="str">
@@ -2630,7 +2645,7 @@
       <x:c r="C16" s="28" t="str">
         <x:v>General ledger / accounting</x:v>
       </x:c>
-      <x:c r="D16" s="46" t="n">
+      <x:c r="D16" s="52" t="n">
         <x:v>46142</x:v>
       </x:c>
       <x:c r="E16" s="28" t="str">
@@ -2656,7 +2671,7 @@
       <x:c r="C17" s="28" t="str">
         <x:v>Bank / treasury</x:v>
       </x:c>
-      <x:c r="D17" s="46" t="n">
+      <x:c r="D17" s="52" t="n">
         <x:v>46142</x:v>
       </x:c>
       <x:c r="E17" s="28" t="str">
@@ -2682,7 +2697,7 @@
       <x:c r="C18" s="28" t="str">
         <x:v>General ledger / accounting</x:v>
       </x:c>
-      <x:c r="D18" s="46" t="n">
+      <x:c r="D18" s="52" t="n">
         <x:v>46142</x:v>
       </x:c>
       <x:c r="E18" s="28" t="str">
@@ -2708,7 +2723,7 @@
       <x:c r="C19" s="28" t="str">
         <x:v>Treasury operations</x:v>
       </x:c>
-      <x:c r="D19" s="46" t="n">
+      <x:c r="D19" s="52" t="n">
         <x:v>46142</x:v>
       </x:c>
       <x:c r="E19" s="28" t="str">
@@ -2734,7 +2749,7 @@
       <x:c r="C20" s="28" t="str">
         <x:v>General ledger / accounting</x:v>
       </x:c>
-      <x:c r="D20" s="46" t="n">
+      <x:c r="D20" s="52" t="n">
         <x:v>46142</x:v>
       </x:c>
       <x:c r="E20" s="28" t="str">
@@ -2760,7 +2775,7 @@
       <x:c r="C21" s="28" t="str">
         <x:v>AP system / AP team</x:v>
       </x:c>
-      <x:c r="D21" s="46" t="n">
+      <x:c r="D21" s="52" t="n">
         <x:v>46142</x:v>
       </x:c>
       <x:c r="E21" s="28" t="str">
@@ -2786,7 +2801,7 @@
       <x:c r="C22" s="28" t="str">
         <x:v>AP system / facilities</x:v>
       </x:c>
-      <x:c r="D22" s="46" t="n">
+      <x:c r="D22" s="52" t="n">
         <x:v>46142</x:v>
       </x:c>
       <x:c r="E22" s="28" t="str">
@@ -2812,7 +2827,7 @@
       <x:c r="C23" s="28" t="str">
         <x:v>Fixed-asset system</x:v>
       </x:c>
-      <x:c r="D23" s="46" t="n">
+      <x:c r="D23" s="52" t="n">
         <x:v>46142</x:v>
       </x:c>
       <x:c r="E23" s="28" t="str">
@@ -2838,7 +2853,7 @@
       <x:c r="C24" s="28" t="str">
         <x:v>Facilities / procurement</x:v>
       </x:c>
-      <x:c r="D24" s="46" t="n">
+      <x:c r="D24" s="52" t="n">
         <x:v>46142</x:v>
       </x:c>
       <x:c r="E24" s="28" t="str">
@@ -2864,7 +2879,7 @@
       <x:c r="C25" s="28" t="str">
         <x:v>Fixed-asset system</x:v>
       </x:c>
-      <x:c r="D25" s="46" t="n">
+      <x:c r="D25" s="52" t="n">
         <x:v>46142</x:v>
       </x:c>
       <x:c r="E25" s="28" t="str">
@@ -2890,7 +2905,7 @@
       <x:c r="C26" s="17" t="str">
         <x:v>Accounting schedules</x:v>
       </x:c>
-      <x:c r="D26" s="47" t="n">
+      <x:c r="D26" s="53" t="n">
         <x:v>46142</x:v>
       </x:c>
       <x:c r="E26" s="17" t="str">
@@ -5943,10 +5958,10 @@
       <x:c r="D5" s="43" t="n">
         <x:v>42800</x:v>
       </x:c>
-      <x:c r="E5" s="28" t="n">
+      <x:c r="E5" s="49" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F5" s="28" t="str">
+      <x:c r="F5" s="49" t="str">
         <x:v>Received</x:v>
       </x:c>
       <x:c r="G5" s="28" t="str">
@@ -5966,10 +5981,10 @@
       <x:c r="D6" s="43" t="n">
         <x:v>86400</x:v>
       </x:c>
-      <x:c r="E6" s="28" t="n">
+      <x:c r="E6" s="49" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F6" s="28" t="str">
+      <x:c r="F6" s="49" t="str">
         <x:v>Received</x:v>
       </x:c>
       <x:c r="G6" s="28" t="str">
@@ -5989,10 +6004,10 @@
       <x:c r="D7" s="43" t="n">
         <x:v>210000</x:v>
       </x:c>
-      <x:c r="E7" s="28" t="n">
+      <x:c r="E7" s="49" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F7" s="28" t="str">
+      <x:c r="F7" s="49" t="str">
         <x:v>Received</x:v>
       </x:c>
       <x:c r="G7" s="28" t="str">
@@ -6012,10 +6027,10 @@
       <x:c r="D8" s="43" t="n">
         <x:v>64500</x:v>
       </x:c>
-      <x:c r="E8" s="28" t="n">
+      <x:c r="E8" s="49" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F8" s="28" t="str">
+      <x:c r="F8" s="49" t="str">
         <x:v>Received</x:v>
       </x:c>
       <x:c r="G8" s="28" t="str">
@@ -6035,10 +6050,10 @@
       <x:c r="D9" s="44" t="n">
         <x:v>1032510</x:v>
       </x:c>
-      <x:c r="E9" s="17" t="n">
+      <x:c r="E9" s="50" t="n">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="F9" s="17" t="str">
+      <x:c r="F9" s="50" t="str">
         <x:v>Mixed</x:v>
       </x:c>
       <x:c r="G9" s="17" t="str">

</xml_diff>